<commit_message>
Add Content Shop home and test campaigns
Automated migration updates generated by Experience Modernization Agent.

Changed files: 55
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-campaigns.report.xlsx
+++ b/tools/importer/reports/import-campaigns.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>index.report.json</t>
+  </si>
+  <si>
+    <t>["hero-campaign","cards-features","cards-features","cards-campaigns","cards-links","tabs"]</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>2026-10-21T09:16:17.431Z</t>
+  </si>
+  <si>
+    <t>Content Shop | Volkswagen</t>
+  </si>
+  <si>
+    <t>http://localhost:8765/index.html</t>
+  </si>
+  <si>
+    <t>campaigns/id-cross.report.json</t>
+  </si>
+  <si>
+    <t>["hero-campaign","columns-info","cards-features","cards-features"]</t>
+  </si>
+  <si>
+    <t>campaigns/id-cross</t>
+  </si>
+  <si>
+    <t>campaign-handbook</t>
+  </si>
+  <si>
+    <t>2026-10-21T09:16:21.995Z</t>
+  </si>
+  <si>
+    <t>ID. Cross — Campaign Handbook | Content Shop</t>
+  </si>
+  <si>
+    <t>http://localhost:8765/campaigns/id-cross.html</t>
+  </si>
+  <si>
     <t>campaigns/id-tiguan.report.json</t>
   </si>
   <si>
@@ -46,19 +91,37 @@
     <t>campaigns/id-tiguan</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>campaigns</t>
   </si>
   <si>
-    <t>2026-10-20T16:30:09.189Z</t>
+    <t>2026-10-21T09:39:35.324Z</t>
   </si>
   <si>
     <t>ID. Tiguan — Instantly Familiar | Campaign overview</t>
   </si>
   <si>
     <t>http://localhost:8765/campaigns/id-tiguan.html</t>
+  </si>
+  <si>
+    <t>fragments/campaign-explore.report.json</t>
+  </si>
+  <si>
+    <t>["cards-links"]</t>
+  </si>
+  <si>
+    <t>fragments/campaign-explore</t>
+  </si>
+  <si>
+    <t>fragment-campaign-explore</t>
+  </si>
+  <si>
+    <t>2026-10-21T09:16:26.988Z</t>
+  </si>
+  <si>
+    <t>Explore more in the Content Shop</t>
+  </si>
+  <si>
+    <t>http://localhost:8765/fragments/campaign-explore.html</t>
   </si>
 </sst>
 </file>
@@ -447,16 +510,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="48" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +571,84 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>